<commit_message>
Simplify label workflows and reorganize dashboard
</commit_message>
<xml_diff>
--- a/data/location-labels.xlsx
+++ b/data/location-labels.xlsx
@@ -421,19 +421,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>A</v>
+        <v>Z</v>
       </c>
       <c r="B2">
+        <v>9</v>
+      </c>
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
       <c r="D2">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E2" t="str">
-        <v>A010215</v>
+        <v>Z090109</v>
       </c>
       <c r="F2">
         <v>1</v>

</xml_diff>